<commit_message>
first try to download
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Devices.xlsx
+++ b/api/src/excelreports/reportTemplates/Devices.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
   <si>
     <t>Code</t>
   </si>
@@ -126,9 +126,6 @@
     <t>Signal loss detected in the amplification curve</t>
   </si>
   <si>
-    <t>Total Tests</t>
-  </si>
-  <si>
     <t>Device Name</t>
   </si>
   <si>
@@ -165,7 +162,28 @@
     <t>&lt;shortName&gt;</t>
   </si>
   <si>
-    <t>&lt;testTotal&gt;</t>
+    <t>Availability</t>
+  </si>
+  <si>
+    <t>&lt;availabilityRate&gt;</t>
+  </si>
+  <si>
+    <t>&lt;issueCategories&gt;</t>
+  </si>
+  <si>
+    <t>Issues</t>
+  </si>
+  <si>
+    <t>This Month</t>
+  </si>
+  <si>
+    <t>&lt;resultCountThisMonth&gt;</t>
+  </si>
+  <si>
+    <t>Last Month</t>
+  </si>
+  <si>
+    <t>&lt;resultCountLastMonth&gt;</t>
   </si>
 </sst>
 </file>
@@ -175,7 +193,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -215,6 +233,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -344,7 +370,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -368,6 +394,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -779,65 +814,88 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="14.75" style="6" customWidth="1"/>
-    <col min="3" max="4" width="14.08203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="12.75" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11" style="6"/>
+    <col min="2" max="3" width="14.75" style="6" customWidth="1"/>
+    <col min="4" max="4" width="29" style="6" customWidth="1"/>
+    <col min="5" max="6" width="14.08203125" style="6" customWidth="1"/>
+    <col min="7" max="8" width="12.75" style="6" customWidth="1"/>
+    <col min="9" max="9" width="11" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+    <row r="4" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="H4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="F5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>46</v>
-      </c>
+      <c r="H5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Cleaning up the code
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Devices.xlsx
+++ b/api/src/excelreports/reportTemplates/Devices.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="57">
   <si>
     <t>Code</t>
   </si>
@@ -184,6 +184,18 @@
   </si>
   <si>
     <t>&lt;resultCountLastMonth&gt;</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>&lt;errorRate&gt;</t>
+  </si>
+  <si>
+    <t>Printed date:</t>
+  </si>
+  <si>
+    <t>&lt;date&gt;</t>
   </si>
 </sst>
 </file>
@@ -814,28 +826,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="3" width="14.75" style="6" customWidth="1"/>
-    <col min="4" max="4" width="29" style="6" customWidth="1"/>
-    <col min="5" max="6" width="14.08203125" style="6" customWidth="1"/>
-    <col min="7" max="8" width="12.75" style="6" customWidth="1"/>
-    <col min="9" max="9" width="11" style="6"/>
+    <col min="2" max="4" width="14.75" style="6" customWidth="1"/>
+    <col min="5" max="5" width="29" style="6" customWidth="1"/>
+    <col min="6" max="7" width="14.08203125" style="6" customWidth="1"/>
+    <col min="8" max="9" width="12.75" style="6" customWidth="1"/>
+    <col min="10" max="10" width="11" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>33</v>
       </c>
@@ -846,25 +866,28 @@
         <v>45</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="J4" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
@@ -874,28 +897,32 @@
       <c r="C5" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
implement feedback on font and corrupt file
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Devices.xlsx
+++ b/api/src/excelreports/reportTemplates/Devices.xlsx
@@ -1,15 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\systemoneid\aspect\api\src\excelreports\reportTemplates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="37920" windowHeight="17240" tabRatio="815"/>
+    <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
@@ -201,7 +196,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
@@ -382,10 +377,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -417,50 +411,56 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -827,102 +827,106 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="4" width="14.75" style="6" customWidth="1"/>
-    <col min="5" max="5" width="29" style="6" customWidth="1"/>
-    <col min="6" max="7" width="14.08203125" style="6" customWidth="1"/>
-    <col min="8" max="9" width="12.75" style="6" customWidth="1"/>
-    <col min="10" max="10" width="11" style="6"/>
+    <col min="2" max="2" width="23.125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.75" style="5" customWidth="1"/>
+    <col min="4" max="4" width="22.5" style="5" customWidth="1"/>
+    <col min="5" max="5" width="40.125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="20.75" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20" style="5" customWidth="1"/>
+    <col min="8" max="8" width="18.75" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18" style="5" customWidth="1"/>
+    <col min="10" max="10" width="16.375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="13" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -938,307 +942,307 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="22" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.08203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.25" customWidth="1"/>
-    <col min="3" max="3" width="100.58203125" customWidth="1"/>
+    <col min="3" max="3" width="100.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8">
+    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
         <v>1001</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8">
+    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
         <v>1002</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8">
+    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
         <v>1004</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8">
+    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
         <v>1005</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8">
+    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
         <v>1006</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8">
+    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
         <v>1007</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8">
+    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
         <v>1017</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8">
+    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
         <v>1018</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8">
+    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
         <v>2003</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="8">
+    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
         <v>2005</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="8">
+    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
         <v>2008</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="8">
+    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
         <v>2009</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="8">
+    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
         <v>2011</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="8">
+    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
         <v>2014</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="8">
+    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7">
         <v>2016</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="8">
+    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
         <v>2018</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="8">
+    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7">
         <v>2022</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="8">
+    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7">
         <v>2025</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8">
+    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7">
         <v>2032</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="8">
+    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
         <v>2034</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="8">
+    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7">
         <v>2037</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8">
+    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7">
         <v>4010</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="8">
+    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7">
         <v>4017</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="8">
+    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7">
         <v>5006</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="8">
+    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7">
         <v>5007</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="8">
+    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="7">
         <v>5011</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>